<commit_message>
Adição do Kaggle usado
</commit_message>
<xml_diff>
--- a/reports/metrics.xlsx
+++ b/reports/metrics.xlsx
@@ -458,7 +458,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -467,25 +467,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.08399999999999989</v>
+        <v>0.3309999999999996</v>
       </c>
       <c r="D2" t="n">
-        <v>0.009119999999999901</v>
+        <v>0.1150449999999997</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0954986910905065</v>
+        <v>0.339182841547151</v>
       </c>
       <c r="F2" t="n">
-        <v>-3.418604651162789</v>
+        <v>-19.45608108108104</v>
       </c>
       <c r="G2" t="n">
-        <v>11.3937356979405</v>
+        <v>7.735655587762444</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -494,19 +494,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.0160531599873629</v>
+        <v>0.0201998075015843</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0003281678547411</v>
+        <v>0.0006390006353153</v>
       </c>
       <c r="E3" t="n">
-        <v>0.018115403797354</v>
+        <v>0.0252784618858693</v>
       </c>
       <c r="F3" t="n">
-        <v>0.8410039463463237</v>
+        <v>0.8863796878884511</v>
       </c>
       <c r="G3" t="n">
-        <v>2.225937156531478</v>
+        <v>0.4729706007766592</v>
       </c>
     </row>
     <row r="4">
@@ -566,7 +566,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -575,25 +575,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.4150000000000002</v>
+        <v>0.2815000000000001</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2674250000000001</v>
+        <v>0.11968625</v>
       </c>
       <c r="E6" t="n">
-        <v>0.5171315113198964</v>
+        <v>0.3459570059993005</v>
       </c>
       <c r="F6" t="n">
-        <v>-1.809086134453784</v>
+        <v>-0.0009220077607544999</v>
       </c>
       <c r="G6" t="n">
-        <v>5.963596037311567</v>
+        <v>1.980006353258783</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -602,25 +602,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.0121744385424804</v>
+        <v>0.0257345768440607</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0002286430890351</v>
+        <v>0.0007574433735019999</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0151209486817169</v>
+        <v>0.0275216891469622</v>
       </c>
       <c r="F7" t="n">
-        <v>0.9975982868798832</v>
+        <v>0.9936655903065664</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1660583474210904</v>
+        <v>0.1781842314046579</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -629,25 +629,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.3309999999999996</v>
+        <v>0.08399999999999989</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1150449999999997</v>
+        <v>0.009119999999999901</v>
       </c>
       <c r="E8" t="n">
-        <v>0.339182841547151</v>
+        <v>0.0954986910905065</v>
       </c>
       <c r="F8" t="n">
-        <v>-19.45608108108104</v>
+        <v>-3.418604651162789</v>
       </c>
       <c r="G8" t="n">
-        <v>7.735655587762444</v>
+        <v>11.3937356979405</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -656,25 +656,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.0201998075015843</v>
+        <v>0.0160531599873629</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0006390006353153</v>
+        <v>0.0003281678547411</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0252784618858693</v>
+        <v>0.018115403797354</v>
       </c>
       <c r="F9" t="n">
-        <v>0.8863796878884511</v>
+        <v>0.8410039463463237</v>
       </c>
       <c r="G9" t="n">
-        <v>0.4729706007766592</v>
+        <v>2.225937156531478</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -683,25 +683,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.2815000000000001</v>
+        <v>0.1930000000000014</v>
       </c>
       <c r="D10" t="n">
-        <v>0.11968625</v>
+        <v>0.0400650000000005</v>
       </c>
       <c r="E10" t="n">
-        <v>0.3459570059993005</v>
+        <v>0.2001624340379596</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.0009220077607544999</v>
+        <v>-13.22762784090916</v>
       </c>
       <c r="G10" t="n">
-        <v>1.980006353258783</v>
+        <v>1.38379200436128</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -710,25 +710,25 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.0257345768440607</v>
+        <v>0.0169408132169763</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0007574433735019999</v>
+        <v>0.0004244514220162</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0275216891469622</v>
+        <v>0.0206022188614771</v>
       </c>
       <c r="F11" t="n">
-        <v>0.9936655903065664</v>
+        <v>0.8492715120681108</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1781842314046579</v>
+        <v>0.1216503216232021</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -737,25 +737,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.1930000000000014</v>
+        <v>0.0351428571428577</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0400650000000005</v>
+        <v>0.0017710204081633</v>
       </c>
       <c r="E12" t="n">
-        <v>0.2001624340379596</v>
+        <v>0.0420834932980058</v>
       </c>
       <c r="F12" t="n">
-        <v>-13.22762784090916</v>
+        <v>-2.304142552543502</v>
       </c>
       <c r="G12" t="n">
-        <v>1.38379200436128</v>
+        <v>0.7956885054955845</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -764,25 +764,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.0169408132169763</v>
+        <v>0.0041119865685454</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0004244514220162</v>
+        <v>1.838776360744211e-05</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0206022188614771</v>
+        <v>0.0042880955688326</v>
       </c>
       <c r="F13" t="n">
-        <v>0.8492715120681108</v>
+        <v>0.9656944708816376</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1216503216232021</v>
+        <v>0.0928850639390624</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -791,25 +791,25 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.0351428571428577</v>
+        <v>0.4150000000000002</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0017710204081633</v>
+        <v>0.2674250000000001</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0420834932980058</v>
+        <v>0.5171315113198964</v>
       </c>
       <c r="F14" t="n">
-        <v>-2.304142552543502</v>
+        <v>-1.809086134453784</v>
       </c>
       <c r="G14" t="n">
-        <v>0.7956885054955845</v>
+        <v>5.963596037311567</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -818,19 +818,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.0041119865685454</v>
+        <v>0.0121744385424804</v>
       </c>
       <c r="D15" t="n">
-        <v>1.838776360744211e-05</v>
+        <v>0.0002286430890351</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0042880955688326</v>
+        <v>0.0151209486817169</v>
       </c>
       <c r="F15" t="n">
-        <v>0.9656944708816376</v>
+        <v>0.9975982868798832</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0928850639390624</v>
+        <v>0.1660583474210904</v>
       </c>
     </row>
     <row r="16">
@@ -890,7 +890,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -899,25 +899,25 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.022</v>
+        <v>0.3220000000000006</v>
       </c>
       <c r="D18" t="n">
-        <v>0.00086</v>
+        <v>0.1405400000000004</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0293257565972303</v>
+        <v>0.3748866495355634</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.0046728971962617</v>
+        <v>-1.464922127122221</v>
       </c>
       <c r="G18" t="n">
-        <v>1.299748849658107</v>
+        <v>3.883937643211752</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -926,19 +926,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.0180151919953163</v>
+        <v>0.0284811627942673</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0003788271562804</v>
+        <v>0.0010961916351326</v>
       </c>
       <c r="E19" t="n">
-        <v>0.0194634826349364</v>
+        <v>0.0331087848634259</v>
       </c>
       <c r="F19" t="n">
-        <v>0.5574449108872995</v>
+        <v>0.9807739645865612</v>
       </c>
       <c r="G19" t="n">
-        <v>1.057797566363949</v>
+        <v>0.3367002630899498</v>
       </c>
     </row>
     <row r="20">
@@ -998,7 +998,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1007,25 +1007,25 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.658</v>
+        <v>0.4580000000000003</v>
       </c>
       <c r="D22" t="n">
-        <v>0.5264599999999999</v>
+        <v>0.2666600000000003</v>
       </c>
       <c r="E22" t="n">
-        <v>0.7255756335489774</v>
+        <v>0.5163913244817347</v>
       </c>
       <c r="F22" t="n">
-        <v>-4.630829126379736</v>
+        <v>-3.68679696287965</v>
       </c>
       <c r="G22" t="n">
-        <v>10.84091254768056</v>
+        <v>10.73018063565718</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1034,25 +1034,25 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.0112474563374046</v>
+        <v>0.0153448164257463</v>
       </c>
       <c r="D23" t="n">
-        <v>0.0003996893957916</v>
+        <v>0.0003402892700773</v>
       </c>
       <c r="E23" t="n">
-        <v>0.019992233386785</v>
+        <v>0.0184469311831888</v>
       </c>
       <c r="F23" t="n">
-        <v>0.9957250642188792</v>
+        <v>0.9940191002868864</v>
       </c>
       <c r="G23" t="n">
-        <v>0.1813839327161096</v>
+        <v>0.3499425926889365</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1061,25 +1061,25 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.1139999999999997</v>
+        <v>0.022</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0158199999999999</v>
+        <v>0.00086</v>
       </c>
       <c r="E24" t="n">
-        <v>0.1257775814682407</v>
+        <v>0.0293257565972303</v>
       </c>
       <c r="F24" t="n">
-        <v>-1.758019525801953</v>
+        <v>-0.0046728971962617</v>
       </c>
       <c r="G24" t="n">
-        <v>2.678654091730834</v>
+        <v>1.299748849658107</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1088,25 +1088,25 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.0125888876911597</v>
+        <v>0.0180151919953163</v>
       </c>
       <c r="D25" t="n">
-        <v>0.0003868531226736</v>
+        <v>0.0003788271562804</v>
       </c>
       <c r="E25" t="n">
-        <v>0.019668582121588</v>
+        <v>0.0194634826349364</v>
       </c>
       <c r="F25" t="n">
-        <v>0.9325569869815804</v>
+        <v>0.5574449108872995</v>
       </c>
       <c r="G25" t="n">
-        <v>0.2911325360887912</v>
+        <v>1.057797566363949</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1115,25 +1115,25 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.1640000000000003</v>
+        <v>0.658</v>
       </c>
       <c r="D26" t="n">
-        <v>0.0319200000000001</v>
+        <v>0.5264599999999999</v>
       </c>
       <c r="E26" t="n">
-        <v>0.1786616914730186</v>
+        <v>0.7255756335489774</v>
       </c>
       <c r="F26" t="n">
-        <v>-5.353503184713395</v>
+        <v>-4.630829126379736</v>
       </c>
       <c r="G26" t="n">
-        <v>6.15779894681447</v>
+        <v>10.84091254768056</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1142,25 +1142,25 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.0064814006181917</v>
+        <v>0.0112474563374046</v>
       </c>
       <c r="D27" t="n">
-        <v>5.958582525590562e-05</v>
+        <v>0.0003996893957916</v>
       </c>
       <c r="E27" t="n">
-        <v>0.0077191855306052</v>
+        <v>0.019992233386785</v>
       </c>
       <c r="F27" t="n">
-        <v>0.9881397640812288</v>
+        <v>0.9957250642188792</v>
       </c>
       <c r="G27" t="n">
-        <v>0.245921672119409</v>
+        <v>0.1813839327161096</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1169,25 +1169,25 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.3220000000000006</v>
+        <v>0.1640000000000003</v>
       </c>
       <c r="D28" t="n">
-        <v>0.1405400000000004</v>
+        <v>0.0319200000000001</v>
       </c>
       <c r="E28" t="n">
-        <v>0.3748866495355634</v>
+        <v>0.1786616914730186</v>
       </c>
       <c r="F28" t="n">
-        <v>-1.464922127122221</v>
+        <v>-5.353503184713395</v>
       </c>
       <c r="G28" t="n">
-        <v>3.883937643211752</v>
+        <v>6.15779894681447</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1196,25 +1196,25 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0.0284811627942673</v>
+        <v>0.0064814006181917</v>
       </c>
       <c r="D29" t="n">
-        <v>0.0010961916351326</v>
+        <v>5.958582525590562e-05</v>
       </c>
       <c r="E29" t="n">
-        <v>0.0331087848634259</v>
+        <v>0.0077191855306052</v>
       </c>
       <c r="F29" t="n">
-        <v>0.9807739645865612</v>
+        <v>0.9881397640812288</v>
       </c>
       <c r="G29" t="n">
-        <v>0.3367002630899498</v>
+        <v>0.245921672119409</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1223,25 +1223,25 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.5999999999999994</v>
+        <v>0.1139999999999997</v>
       </c>
       <c r="D30" t="n">
-        <v>0.4529999999999993</v>
+        <v>0.0158199999999999</v>
       </c>
       <c r="E30" t="n">
-        <v>0.6730527468185531</v>
+        <v>0.1257775814682407</v>
       </c>
       <c r="F30" t="n">
-        <v>-3.870967741935478</v>
+        <v>-1.758019525801953</v>
       </c>
       <c r="G30" t="n">
-        <v>8.880724578126173</v>
+        <v>2.678654091730834</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1250,25 +1250,25 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.0281213648827217</v>
+        <v>0.0125888876911597</v>
       </c>
       <c r="D31" t="n">
-        <v>0.0010277804435704</v>
+        <v>0.0003868531226736</v>
       </c>
       <c r="E31" t="n">
-        <v>0.0320590150124808</v>
+        <v>0.019668582121588</v>
       </c>
       <c r="F31" t="n">
-        <v>0.9889485973809626</v>
+        <v>0.9325569869815804</v>
       </c>
       <c r="G31" t="n">
-        <v>0.4147634566532974</v>
+        <v>0.2911325360887912</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1277,25 +1277,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.4580000000000003</v>
+        <v>0.5999999999999994</v>
       </c>
       <c r="D32" t="n">
-        <v>0.2666600000000003</v>
+        <v>0.4529999999999993</v>
       </c>
       <c r="E32" t="n">
-        <v>0.5163913244817347</v>
+        <v>0.6730527468185531</v>
       </c>
       <c r="F32" t="n">
-        <v>-3.68679696287965</v>
+        <v>-3.870967741935478</v>
       </c>
       <c r="G32" t="n">
-        <v>10.73018063565718</v>
+        <v>8.880724578126173</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1304,25 +1304,25 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0.0153448164257463</v>
+        <v>0.0281213648827217</v>
       </c>
       <c r="D33" t="n">
-        <v>0.0003402892700773</v>
+        <v>0.0010277804435704</v>
       </c>
       <c r="E33" t="n">
-        <v>0.0184469311831888</v>
+        <v>0.0320590150124808</v>
       </c>
       <c r="F33" t="n">
-        <v>0.9940191002868864</v>
+        <v>0.9889485973809626</v>
       </c>
       <c r="G33" t="n">
-        <v>0.3499425926889365</v>
+        <v>0.4147634566532974</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Israel</t>
+          <t>Iran</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1331,25 +1331,25 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0.4859999999999994</v>
+        <v>0.8</v>
       </c>
       <c r="D34" t="n">
-        <v>0.2925799999999993</v>
+        <v>0.7237200000000001</v>
       </c>
       <c r="E34" t="n">
-        <v>0.5409066462893568</v>
+        <v>0.8507173443629794</v>
       </c>
       <c r="F34" t="n">
-        <v>-4.189060726447212</v>
+        <v>-16.18886566596994</v>
       </c>
       <c r="G34" t="n">
-        <v>8.84985833402517</v>
+        <v>9.223668237956668</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Israel</t>
+          <t>Iran</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1358,25 +1358,25 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.0137106719488279</v>
+        <v>0.0067609848853393</v>
       </c>
       <c r="D35" t="n">
-        <v>0.0002275310968075</v>
+        <v>5.799028666439593e-05</v>
       </c>
       <c r="E35" t="n">
-        <v>0.0150841339429073</v>
+        <v>0.0076151353674373</v>
       </c>
       <c r="F35" t="n">
-        <v>0.9959646159050872</v>
+        <v>0.9986226893724016</v>
       </c>
       <c r="G35" t="n">
-        <v>0.2482522049268466</v>
+        <v>0.07785225430370619</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Iran</t>
+          <t>India</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1385,25 +1385,25 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0.8</v>
+        <v>0.1999999999999998</v>
       </c>
       <c r="D36" t="n">
-        <v>0.7237200000000001</v>
+        <v>0.0478399999999999</v>
       </c>
       <c r="E36" t="n">
-        <v>0.8507173443629794</v>
+        <v>0.2187235698318768</v>
       </c>
       <c r="F36" t="n">
-        <v>-16.18886566596994</v>
+        <v>-5.102040816326523</v>
       </c>
       <c r="G36" t="n">
-        <v>9.223668237956668</v>
+        <v>9.77434397771882</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Iran</t>
+          <t>India</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1412,25 +1412,25 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0.0067609848853393</v>
+        <v>0.005578911634433</v>
       </c>
       <c r="D37" t="n">
-        <v>5.799028666439593e-05</v>
+        <v>6.145303781597753e-05</v>
       </c>
       <c r="E37" t="n">
-        <v>0.0076151353674373</v>
+        <v>0.007839198799365701</v>
       </c>
       <c r="F37" t="n">
-        <v>0.9986226893724016</v>
+        <v>0.9921616023193908</v>
       </c>
       <c r="G37" t="n">
-        <v>0.07785225430370619</v>
+        <v>0.2775392800587057</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1439,25 +1439,25 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0.1999999999999998</v>
+        <v>0.372</v>
       </c>
       <c r="D38" t="n">
-        <v>0.0478399999999999</v>
+        <v>0.15596</v>
       </c>
       <c r="E38" t="n">
-        <v>0.2187235698318768</v>
+        <v>0.3949177129479</v>
       </c>
       <c r="F38" t="n">
-        <v>-5.102040816326523</v>
+        <v>-7.873463814292235</v>
       </c>
       <c r="G38" t="n">
-        <v>9.77434397771882</v>
+        <v>7.241533422227336</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1466,19 +1466,19 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0.005578911634433</v>
+        <v>0.0490261069519627</v>
       </c>
       <c r="D39" t="n">
-        <v>6.145303781597753e-05</v>
+        <v>0.003146052781261</v>
       </c>
       <c r="E39" t="n">
-        <v>0.007839198799365701</v>
+        <v>0.0560896851592259</v>
       </c>
       <c r="F39" t="n">
-        <v>0.9921616023193908</v>
+        <v>0.8210029141294325</v>
       </c>
       <c r="G39" t="n">
-        <v>0.2775392800587057</v>
+        <v>0.9529755956440644</v>
       </c>
     </row>
     <row r="40">
@@ -1538,7 +1538,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1547,25 +1547,25 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0.1906666666666662</v>
+        <v>0.1279999999999999</v>
       </c>
       <c r="D42" t="n">
-        <v>0.046391111111111</v>
+        <v>0.02324</v>
       </c>
       <c r="E42" t="n">
-        <v>0.2153859584817707</v>
+        <v>0.152446712001276</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.0046585046585054</v>
+        <v>-0.1100496752006123</v>
       </c>
       <c r="G42" t="n">
-        <v>1.344403599331216</v>
+        <v>2.569093836961529</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1574,25 +1574,25 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0.0070652549191247</v>
+        <v>0.0113241631290858</v>
       </c>
       <c r="D43" t="n">
-        <v>6.963056293923933e-05</v>
+        <v>0.0001986890078835</v>
       </c>
       <c r="E43" t="n">
-        <v>0.008344492970770501</v>
+        <v>0.0140957088464371</v>
       </c>
       <c r="F43" t="n">
-        <v>0.9984920616134088</v>
+        <v>0.9905096958404888</v>
       </c>
       <c r="G43" t="n">
-        <v>0.0493542840872781</v>
+        <v>0.2245647611556721</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1601,25 +1601,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0.1279999999999999</v>
+        <v>0.5880000000000006</v>
       </c>
       <c r="D44" t="n">
-        <v>0.02324</v>
+        <v>0.4414400000000008</v>
       </c>
       <c r="E44" t="n">
-        <v>0.152446712001276</v>
+        <v>0.6644095122738692</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.1100496752006123</v>
+        <v>-3.612940979769277</v>
       </c>
       <c r="G44" t="n">
-        <v>2.569093836961529</v>
+        <v>7.797402461964853</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1628,25 +1628,25 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0.0113241631290858</v>
+        <v>0.0405819675822938</v>
       </c>
       <c r="D45" t="n">
-        <v>0.0001986890078835</v>
+        <v>0.0017851968954592</v>
       </c>
       <c r="E45" t="n">
-        <v>0.0140957088464371</v>
+        <v>0.042251590448872</v>
       </c>
       <c r="F45" t="n">
-        <v>0.9905096958404888</v>
+        <v>0.9813451252355456</v>
       </c>
       <c r="G45" t="n">
-        <v>0.2245647611556721</v>
+        <v>0.5318021691491214</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Israel</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1655,25 +1655,25 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0.372</v>
+        <v>0.4859999999999994</v>
       </c>
       <c r="D46" t="n">
-        <v>0.15596</v>
+        <v>0.2925799999999993</v>
       </c>
       <c r="E46" t="n">
-        <v>0.3949177129479</v>
+        <v>0.5409066462893568</v>
       </c>
       <c r="F46" t="n">
-        <v>-7.873463814292235</v>
+        <v>-4.189060726447212</v>
       </c>
       <c r="G46" t="n">
-        <v>7.241533422227336</v>
+        <v>8.84985833402517</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Israel</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1682,25 +1682,25 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0.0490261069519627</v>
+        <v>0.0137106719488279</v>
       </c>
       <c r="D47" t="n">
-        <v>0.003146052781261</v>
+        <v>0.0002275310968075</v>
       </c>
       <c r="E47" t="n">
-        <v>0.0560896851592259</v>
+        <v>0.0150841339429073</v>
       </c>
       <c r="F47" t="n">
-        <v>0.8210029141294325</v>
+        <v>0.9959646159050872</v>
       </c>
       <c r="G47" t="n">
-        <v>0.9529755956440644</v>
+        <v>0.2482522049268466</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1709,25 +1709,25 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0.5880000000000006</v>
+        <v>0.1906666666666662</v>
       </c>
       <c r="D48" t="n">
-        <v>0.4414400000000008</v>
+        <v>0.046391111111111</v>
       </c>
       <c r="E48" t="n">
-        <v>0.6644095122738692</v>
+        <v>0.2153859584817707</v>
       </c>
       <c r="F48" t="n">
-        <v>-3.612940979769277</v>
+        <v>-0.0046585046585054</v>
       </c>
       <c r="G48" t="n">
-        <v>7.797402461964853</v>
+        <v>1.344403599331216</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1736,25 +1736,25 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0.0405819675822938</v>
+        <v>0.0070652549191247</v>
       </c>
       <c r="D49" t="n">
-        <v>0.0017851968954592</v>
+        <v>6.963056293923933e-05</v>
       </c>
       <c r="E49" t="n">
-        <v>0.042251590448872</v>
+        <v>0.008344492970770501</v>
       </c>
       <c r="F49" t="n">
-        <v>0.9813451252355456</v>
+        <v>0.9984920616134088</v>
       </c>
       <c r="G49" t="n">
-        <v>0.5318021691491214</v>
+        <v>0.0493542840872781</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Kuwait</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1763,25 +1763,25 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0.0419999999999999</v>
+        <v>0.5573333333333323</v>
       </c>
       <c r="D50" t="n">
-        <v>0.0023799999999999</v>
+        <v>0.5403955555555543</v>
       </c>
       <c r="E50" t="n">
-        <v>0.0487852436706018</v>
+        <v>0.7351160150313379</v>
       </c>
       <c r="F50" t="n">
-        <v>-2.863636363636358</v>
+        <v>-1.06933935129873</v>
       </c>
       <c r="G50" t="n">
-        <v>9.220531537974626</v>
+        <v>2.453464384057162</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Kuwait</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1790,25 +1790,25 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0.015056027364533</v>
+        <v>0.0930518040838649</v>
       </c>
       <c r="D51" t="n">
-        <v>0.0002733533713564</v>
+        <v>0.0094577636203557</v>
       </c>
       <c r="E51" t="n">
-        <v>0.016533401687387</v>
+        <v>0.09725103403232151</v>
       </c>
       <c r="F51" t="n">
-        <v>0.5562445270186797</v>
+        <v>0.9637833393822728</v>
       </c>
       <c r="G51" t="n">
-        <v>3.335498736964023</v>
+        <v>0.4142450435641097</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Kuwait</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1817,25 +1817,25 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0.5573333333333323</v>
+        <v>0.124</v>
       </c>
       <c r="D52" t="n">
-        <v>0.5403955555555543</v>
+        <v>0.01904</v>
       </c>
       <c r="E52" t="n">
-        <v>0.7351160150313379</v>
+        <v>0.1379855064852828</v>
       </c>
       <c r="F52" t="n">
-        <v>-1.06933935129873</v>
+        <v>-4.196506550218334</v>
       </c>
       <c r="G52" t="n">
-        <v>2.453464384057162</v>
+        <v>5.95468115678282</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Kuwait</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1844,19 +1844,19 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0.0930518040838649</v>
+        <v>0.0061897086728856</v>
       </c>
       <c r="D53" t="n">
-        <v>0.0094577636203557</v>
+        <v>6.792816137230078e-05</v>
       </c>
       <c r="E53" t="n">
-        <v>0.09725103403232151</v>
+        <v>0.0082418542435729</v>
       </c>
       <c r="F53" t="n">
-        <v>0.9637833393822728</v>
+        <v>0.981460654647298</v>
       </c>
       <c r="G53" t="n">
-        <v>0.4142450435641097</v>
+        <v>0.2996470704291382</v>
       </c>
     </row>
     <row r="54">
@@ -1970,7 +1970,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1979,25 +1979,25 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>0.044</v>
+        <v>0.840000000000001</v>
       </c>
       <c r="D58" t="n">
-        <v>0.00228</v>
+        <v>0.7466800000000016</v>
       </c>
       <c r="E58" t="n">
-        <v>0.0477493455452533</v>
+        <v>0.8641064749207713</v>
       </c>
       <c r="F58" t="n">
-        <v>-5.627906976744185</v>
+        <v>-17.17624148003895</v>
       </c>
       <c r="G58" t="n">
-        <v>6.857982295482302</v>
+        <v>11.60891078136201</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2006,25 +2006,25 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0.0090762926550822</v>
+        <v>0.0188964841009362</v>
       </c>
       <c r="D59" t="n">
-        <v>0.0001023074499689</v>
+        <v>0.0005033936626767</v>
       </c>
       <c r="E59" t="n">
-        <v>0.0101147145273093</v>
+        <v>0.0224364360511363</v>
       </c>
       <c r="F59" t="n">
-        <v>0.7025946221832473</v>
+        <v>0.9877460160010534</v>
       </c>
       <c r="G59" t="n">
-        <v>1.431185781735938</v>
+        <v>0.2574361962979577</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2033,25 +2033,25 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>0.840000000000001</v>
+        <v>0.044</v>
       </c>
       <c r="D60" t="n">
-        <v>0.7466800000000016</v>
+        <v>0.00228</v>
       </c>
       <c r="E60" t="n">
-        <v>0.8641064749207713</v>
+        <v>0.0477493455452533</v>
       </c>
       <c r="F60" t="n">
-        <v>-17.17624148003895</v>
+        <v>-5.627906976744185</v>
       </c>
       <c r="G60" t="n">
-        <v>11.60891078136201</v>
+        <v>6.857982295482302</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2060,25 +2060,25 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>0.0188964841009362</v>
+        <v>0.0090762926550822</v>
       </c>
       <c r="D61" t="n">
-        <v>0.0005033936626767</v>
+        <v>0.0001023074499689</v>
       </c>
       <c r="E61" t="n">
-        <v>0.0224364360511363</v>
+        <v>0.0101147145273093</v>
       </c>
       <c r="F61" t="n">
-        <v>0.9877460160010534</v>
+        <v>0.7025946221832473</v>
       </c>
       <c r="G61" t="n">
-        <v>0.2574361962979577</v>
+        <v>1.431185781735938</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2087,25 +2087,25 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>0.3319999999999997</v>
+        <v>0.0419999999999999</v>
       </c>
       <c r="D62" t="n">
-        <v>0.1710399999999997</v>
+        <v>0.0023799999999999</v>
       </c>
       <c r="E62" t="n">
-        <v>0.4135698248180103</v>
+        <v>0.0487852436706018</v>
       </c>
       <c r="F62" t="n">
-        <v>-1.812417784793473</v>
+        <v>-2.863636363636358</v>
       </c>
       <c r="G62" t="n">
-        <v>4.334787368628502</v>
+        <v>9.220531537974626</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2114,25 +2114,25 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>0.0100597391605177</v>
+        <v>0.015056027364533</v>
       </c>
       <c r="D63" t="n">
-        <v>0.0001631857439114</v>
+        <v>0.0002733533713564</v>
       </c>
       <c r="E63" t="n">
-        <v>0.0127744175566406</v>
+        <v>0.016533401687387</v>
       </c>
       <c r="F63" t="n">
-        <v>0.9973167300724908</v>
+        <v>0.5562445270186797</v>
       </c>
       <c r="G63" t="n">
-        <v>0.1276506367000497</v>
+        <v>3.335498736964023</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2141,25 +2141,25 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>0.124</v>
+        <v>0.3319999999999997</v>
       </c>
       <c r="D64" t="n">
-        <v>0.01904</v>
+        <v>0.1710399999999997</v>
       </c>
       <c r="E64" t="n">
-        <v>0.1379855064852828</v>
+        <v>0.4135698248180103</v>
       </c>
       <c r="F64" t="n">
-        <v>-4.196506550218334</v>
+        <v>-1.812417784793473</v>
       </c>
       <c r="G64" t="n">
-        <v>5.95468115678282</v>
+        <v>4.334787368628502</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2168,25 +2168,25 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>0.0061897086728856</v>
+        <v>0.0100597391605177</v>
       </c>
       <c r="D65" t="n">
-        <v>6.792816137230078e-05</v>
+        <v>0.0001631857439114</v>
       </c>
       <c r="E65" t="n">
-        <v>0.0082418542435729</v>
+        <v>0.0127744175566406</v>
       </c>
       <c r="F65" t="n">
-        <v>0.981460654647298</v>
+        <v>0.9973167300724908</v>
       </c>
       <c r="G65" t="n">
-        <v>0.2996470704291382</v>
+        <v>0.1276506367000497</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2195,25 +2195,25 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>0.2080000000000003</v>
+        <v>0.1579999999999999</v>
       </c>
       <c r="D66" t="n">
-        <v>0.0662000000000002</v>
+        <v>0.0294599999999999</v>
       </c>
       <c r="E66" t="n">
-        <v>0.2572936066053726</v>
+        <v>0.1716391563717323</v>
       </c>
       <c r="F66" t="n">
-        <v>-0.1465983095469052</v>
+        <v>-5.552491103202848</v>
       </c>
       <c r="G66" t="n">
-        <v>2.570431270812694</v>
+        <v>10.56984198478326</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2222,25 +2222,25 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>0.0094485018040138</v>
+        <v>0.0116899247585407</v>
       </c>
       <c r="D67" t="n">
-        <v>0.000167068198356</v>
+        <v>0.0001566927408099</v>
       </c>
       <c r="E67" t="n">
-        <v>0.0129254863876018</v>
+        <v>0.0125176971048983</v>
       </c>
       <c r="F67" t="n">
-        <v>0.9971063426916296</v>
+        <v>0.9651484117415524</v>
       </c>
       <c r="G67" t="n">
-        <v>0.1197552022575391</v>
+        <v>0.7860506446376264</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Qatar</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2249,25 +2249,25 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0.1579999999999999</v>
+        <v>0.7460000000000008</v>
       </c>
       <c r="D68" t="n">
-        <v>0.0294599999999999</v>
+        <v>1.30698</v>
       </c>
       <c r="E68" t="n">
-        <v>0.1716391563717323</v>
+        <v>1.143232259866734</v>
       </c>
       <c r="F68" t="n">
-        <v>-5.552491103202848</v>
+        <v>0.0076503960347923</v>
       </c>
       <c r="G68" t="n">
-        <v>10.56984198478326</v>
+        <v>1.90555298762894</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Qatar</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2276,19 +2276,19 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0.0116899247585407</v>
+        <v>0.2582100811261497</v>
       </c>
       <c r="D69" t="n">
-        <v>0.0001566927408099</v>
+        <v>0.08191992728623559</v>
       </c>
       <c r="E69" t="n">
-        <v>0.0125176971048983</v>
+        <v>0.2862165740942262</v>
       </c>
       <c r="F69" t="n">
-        <v>0.9651484117415524</v>
+        <v>0.9378007257958388</v>
       </c>
       <c r="G69" t="n">
-        <v>0.7860506446376264</v>
+        <v>0.6791488306746781</v>
       </c>
     </row>
     <row r="70">
@@ -2348,7 +2348,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Qatar</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2357,25 +2357,25 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>0.7460000000000008</v>
+        <v>0.2080000000000003</v>
       </c>
       <c r="D72" t="n">
-        <v>1.30698</v>
+        <v>0.0662000000000002</v>
       </c>
       <c r="E72" t="n">
-        <v>1.143232259866734</v>
+        <v>0.2572936066053726</v>
       </c>
       <c r="F72" t="n">
-        <v>0.0076503960347923</v>
+        <v>-0.1465983095469052</v>
       </c>
       <c r="G72" t="n">
-        <v>1.90555298762894</v>
+        <v>2.570431270812694</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Qatar</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2384,25 +2384,25 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>0.2582100811261497</v>
+        <v>0.0094485018040138</v>
       </c>
       <c r="D73" t="n">
-        <v>0.08191992728623559</v>
+        <v>0.000167068198356</v>
       </c>
       <c r="E73" t="n">
-        <v>0.2862165740942262</v>
+        <v>0.0129254863876018</v>
       </c>
       <c r="F73" t="n">
-        <v>0.9378007257958388</v>
+        <v>0.9971063426916296</v>
       </c>
       <c r="G73" t="n">
-        <v>0.6791488306746781</v>
+        <v>0.1197552022575391</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Russia</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2411,25 +2411,25 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>0.4259999999999998</v>
+        <v>0.4779999999999997</v>
       </c>
       <c r="D74" t="n">
-        <v>0.2031799999999998</v>
+        <v>0.2704199999999996</v>
       </c>
       <c r="E74" t="n">
-        <v>0.4507549223247594</v>
+        <v>0.5200192304136451</v>
       </c>
       <c r="F74" t="n">
-        <v>-0.9908677588774796</v>
+        <v>-1.172117979694125</v>
       </c>
       <c r="G74" t="n">
-        <v>2.428207462988676</v>
+        <v>3.821242323173678</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Russia</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2438,25 +2438,25 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>0.0280326833865423</v>
+        <v>0.0530260740977809</v>
       </c>
       <c r="D75" t="n">
-        <v>0.0013035150458352</v>
+        <v>0.0037859433390974</v>
       </c>
       <c r="E75" t="n">
-        <v>0.0361042247643582</v>
+        <v>0.0615300198203887</v>
       </c>
       <c r="F75" t="n">
-        <v>0.987227453105792</v>
+        <v>0.969589839520166</v>
       </c>
       <c r="G75" t="n">
-        <v>0.1589053841712803</v>
+        <v>0.4223986483954648</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2465,25 +2465,25 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>0.3979999999999997</v>
+        <v>0.4259999999999998</v>
       </c>
       <c r="D76" t="n">
-        <v>0.1706599999999997</v>
+        <v>0.2031799999999998</v>
       </c>
       <c r="E76" t="n">
-        <v>0.4131101548013553</v>
+        <v>0.4507549223247594</v>
       </c>
       <c r="F76" t="n">
-        <v>-2.797845825173569</v>
+        <v>-0.9908677588774796</v>
       </c>
       <c r="G76" t="n">
-        <v>3.516244929353495</v>
+        <v>2.428207462988676</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2492,19 +2492,19 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>0.0200098794718698</v>
+        <v>0.0280326833865423</v>
       </c>
       <c r="D77" t="n">
-        <v>0.0004392484901971</v>
+        <v>0.0013035150458352</v>
       </c>
       <c r="E77" t="n">
-        <v>0.0209582558958785</v>
+        <v>0.0361042247643582</v>
       </c>
       <c r="F77" t="n">
-        <v>0.9902250202466368</v>
+        <v>0.987227453105792</v>
       </c>
       <c r="G77" t="n">
-        <v>0.176472782923132</v>
+        <v>0.1589053841712803</v>
       </c>
     </row>
     <row r="78">
@@ -2564,7 +2564,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2573,25 +2573,25 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>0.4779999999999997</v>
+        <v>0.3979999999999997</v>
       </c>
       <c r="D80" t="n">
-        <v>0.2704199999999996</v>
+        <v>0.1706599999999997</v>
       </c>
       <c r="E80" t="n">
-        <v>0.5200192304136451</v>
+        <v>0.4131101548013553</v>
       </c>
       <c r="F80" t="n">
-        <v>-1.172117979694125</v>
+        <v>-2.797845825173569</v>
       </c>
       <c r="G80" t="n">
-        <v>3.821242323173678</v>
+        <v>3.516244929353495</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2600,25 +2600,25 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>0.0530260740977809</v>
+        <v>0.0200098794718698</v>
       </c>
       <c r="D81" t="n">
-        <v>0.0037859433390974</v>
+        <v>0.0004392484901971</v>
       </c>
       <c r="E81" t="n">
-        <v>0.0615300198203887</v>
+        <v>0.0209582558958785</v>
       </c>
       <c r="F81" t="n">
-        <v>0.969589839520166</v>
+        <v>0.9902250202466368</v>
       </c>
       <c r="G81" t="n">
-        <v>0.4223986483954648</v>
+        <v>0.176472782923132</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2627,25 +2627,25 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>0.3159999999999998</v>
+        <v>0.1330000000000001</v>
       </c>
       <c r="D82" t="n">
-        <v>0.1177199999999998</v>
+        <v>0.022215</v>
       </c>
       <c r="E82" t="n">
-        <v>0.3431034829318988</v>
+        <v>0.1490469724617043</v>
       </c>
       <c r="F82" t="n">
-        <v>-2.627064333251162</v>
+        <v>-0.732298814722403</v>
       </c>
       <c r="G82" t="n">
-        <v>5.687255197120349</v>
+        <v>2.850275697126901</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2654,25 +2654,25 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>0.0204848844193488</v>
+        <v>0.0453764014803111</v>
       </c>
       <c r="D83" t="n">
-        <v>0.0005289507243558</v>
+        <v>0.002517157493137</v>
       </c>
       <c r="E83" t="n">
-        <v>0.0229989287653979</v>
+        <v>0.0501712815576503</v>
       </c>
       <c r="F83" t="n">
-        <v>0.9837025288280796</v>
+        <v>0.8037151050267443</v>
       </c>
       <c r="G83" t="n">
-        <v>0.3733166965414429</v>
+        <v>0.9758820899495414</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2681,25 +2681,25 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>0.1330000000000001</v>
+        <v>0.0899999999999998</v>
       </c>
       <c r="D84" t="n">
-        <v>0.022215</v>
+        <v>0.0100199999999999</v>
       </c>
       <c r="E84" t="n">
-        <v>0.1490469724617043</v>
+        <v>0.1000999500499375</v>
       </c>
       <c r="F84" t="n">
-        <v>-0.732298814722403</v>
+        <v>-0.2136627906976722</v>
       </c>
       <c r="G84" t="n">
-        <v>2.850275697126901</v>
+        <v>2.022377291062895</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2708,19 +2708,19 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>0.0453764014803111</v>
+        <v>0.0193409166073452</v>
       </c>
       <c r="D85" t="n">
-        <v>0.002517157493137</v>
+        <v>0.0004741066822955</v>
       </c>
       <c r="E85" t="n">
-        <v>0.0501712815576503</v>
+        <v>0.0217739909592965</v>
       </c>
       <c r="F85" t="n">
-        <v>0.8037151050267443</v>
+        <v>0.9425742875126544</v>
       </c>
       <c r="G85" t="n">
-        <v>0.9758820899495414</v>
+        <v>0.437584062413683</v>
       </c>
     </row>
     <row r="86">
@@ -2780,7 +2780,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2789,25 +2789,25 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>0.2459999999999993</v>
+        <v>0.3159999999999998</v>
       </c>
       <c r="D88" t="n">
-        <v>0.0679399999999997</v>
+        <v>0.1177199999999998</v>
       </c>
       <c r="E88" t="n">
-        <v>0.2606530260710581</v>
+        <v>0.3431034829318988</v>
       </c>
       <c r="F88" t="n">
-        <v>-0.013424821002385</v>
+        <v>-2.627064333251162</v>
       </c>
       <c r="G88" t="n">
-        <v>1.720155846652194</v>
+        <v>5.687255197120349</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2816,25 +2816,25 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>0.0240742808719822</v>
+        <v>0.0204848844193488</v>
       </c>
       <c r="D89" t="n">
-        <v>0.0012166790620129</v>
+        <v>0.0005289507243558</v>
       </c>
       <c r="E89" t="n">
-        <v>0.0348809269087411</v>
+        <v>0.0229989287653979</v>
       </c>
       <c r="F89" t="n">
-        <v>0.9818514459723606</v>
+        <v>0.9837025288280796</v>
       </c>
       <c r="G89" t="n">
-        <v>0.170459054023749</v>
+        <v>0.3733166965414429</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2843,25 +2843,25 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>0.0899999999999998</v>
+        <v>0.5920000000000003</v>
       </c>
       <c r="D90" t="n">
-        <v>0.0100199999999999</v>
+        <v>0.4334400000000005</v>
       </c>
       <c r="E90" t="n">
-        <v>0.1000999500499375</v>
+        <v>0.6583616027685701</v>
       </c>
       <c r="F90" t="n">
-        <v>-0.2136627906976722</v>
+        <v>-6.958284371327848</v>
       </c>
       <c r="G90" t="n">
-        <v>2.022377291062895</v>
+        <v>13.97680555154674</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2870,19 +2870,19 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>0.0193409166073452</v>
+        <v>0.0170348122768711</v>
       </c>
       <c r="D91" t="n">
-        <v>0.0004741066822955</v>
+        <v>0.0004025733106673</v>
       </c>
       <c r="E91" t="n">
-        <v>0.0217739909592965</v>
+        <v>0.020064229630547</v>
       </c>
       <c r="F91" t="n">
-        <v>0.9425742875126544</v>
+        <v>0.9926084512583117</v>
       </c>
       <c r="G91" t="n">
-        <v>0.437584062413683</v>
+        <v>0.4033249679561881</v>
       </c>
     </row>
     <row r="92">
@@ -2996,7 +2996,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3005,25 +3005,25 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>0.5920000000000003</v>
+        <v>0.2459999999999993</v>
       </c>
       <c r="D96" t="n">
-        <v>0.4334400000000005</v>
+        <v>0.0679399999999997</v>
       </c>
       <c r="E96" t="n">
-        <v>0.6583616027685701</v>
+        <v>0.2606530260710581</v>
       </c>
       <c r="F96" t="n">
-        <v>-6.958284371327848</v>
+        <v>-0.013424821002385</v>
       </c>
       <c r="G96" t="n">
-        <v>13.97680555154674</v>
+        <v>1.720155846652194</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -3032,25 +3032,25 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>0.0170348122768711</v>
+        <v>0.0240742808719822</v>
       </c>
       <c r="D97" t="n">
-        <v>0.0004025733106673</v>
+        <v>0.0012166790620129</v>
       </c>
       <c r="E97" t="n">
-        <v>0.020064229630547</v>
+        <v>0.0348809269087411</v>
       </c>
       <c r="F97" t="n">
-        <v>0.9926084512583117</v>
+        <v>0.9818514459723606</v>
       </c>
       <c r="G97" t="n">
-        <v>0.4033249679561881</v>
+        <v>0.170459054023749</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Venezuela</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -3059,25 +3059,25 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>0.2619999999999999</v>
+        <v>0.702</v>
       </c>
       <c r="D98" t="n">
-        <v>0.07093999999999991</v>
+        <v>0.6020199999999999</v>
       </c>
       <c r="E98" t="n">
-        <v>0.2663456400994767</v>
+        <v>0.7758994780253431</v>
       </c>
       <c r="F98" t="n">
-        <v>-29.89721254355398</v>
+        <v>-4.512196015235864</v>
       </c>
       <c r="G98" t="n">
-        <v>5.942769612116751</v>
+        <v>16.17998633780347</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Venezuela</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -3086,25 +3086,25 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>0.009434009093816901</v>
+        <v>0.0208114173821286</v>
       </c>
       <c r="D99" t="n">
-        <v>0.0001387488402483</v>
+        <v>0.0006651118944544</v>
       </c>
       <c r="E99" t="n">
-        <v>0.0117791697605728</v>
+        <v>0.0257897633656165</v>
       </c>
       <c r="F99" t="n">
-        <v>0.9395693204493062</v>
+        <v>0.9939101240252848</v>
       </c>
       <c r="G99" t="n">
-        <v>0.2132629922243628</v>
+        <v>0.4755997544123395</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Venezuela</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3113,25 +3113,25 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>0.702</v>
+        <v>0.2619999999999999</v>
       </c>
       <c r="D100" t="n">
-        <v>0.6020199999999999</v>
+        <v>0.07093999999999991</v>
       </c>
       <c r="E100" t="n">
-        <v>0.7758994780253431</v>
+        <v>0.2663456400994767</v>
       </c>
       <c r="F100" t="n">
-        <v>-4.512196015235864</v>
+        <v>-29.89721254355398</v>
       </c>
       <c r="G100" t="n">
-        <v>16.17998633780347</v>
+        <v>5.942769612116751</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Venezuela</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3140,19 +3140,19 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>0.0208114173821286</v>
+        <v>0.009434009093816901</v>
       </c>
       <c r="D101" t="n">
-        <v>0.0006651118944544</v>
+        <v>0.0001387488402483</v>
       </c>
       <c r="E101" t="n">
-        <v>0.0257897633656165</v>
+        <v>0.0117791697605728</v>
       </c>
       <c r="F101" t="n">
-        <v>0.9939101240252848</v>
+        <v>0.9395693204493062</v>
       </c>
       <c r="G101" t="n">
-        <v>0.4755997544123395</v>
+        <v>0.2132629922243628</v>
       </c>
     </row>
   </sheetData>

</xml_diff>